<commit_message>
Actualizacion automatica 2026-09-17 17:35 UTC
</commit_message>
<xml_diff>
--- a/data/50001449 -  Itaberaba Extracción.xlsx
+++ b/data/50001449 -  Itaberaba Extracción.xlsx
@@ -3296,7 +3296,7 @@
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="5">
-        <v>46258.65920591435</v>
+        <v>46282.16941618056</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>71</v>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="C41" s="10"/>
       <c r="D41" s="9">
-        <v>46275.141257511576</v>
+        <v>46282.169413958334</v>
       </c>
       <c r="E41" s="10" t="s">
         <v>144</v>

</xml_diff>